<commit_message>
Fixed country data for spanish template
</commit_message>
<xml_diff>
--- a/src/R/risk_cut_offs.xlsx
+++ b/src/R/risk_cut_offs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivermazariegos/Sites/polio-risk/src/R/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5aee5c5b004427f/Documents/polio-risk-assessment/src/R/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2130697D-5267-FA46-BBC8-B56D5280EFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{2130697D-5267-FA46-BBC8-B56D5280EFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FC6EF47-E285-4DF9-BF1B-3A10E9C6B2F5}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1820" windowWidth="24500" windowHeight="17240" xr2:uid="{5C1FCA5E-1AE1-4E42-BC50-0F3DA39A67C4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{5C1FCA5E-1AE1-4E42-BC50-0F3DA39A67C4}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet_cut_off" sheetId="2" r:id="rId1"/>
@@ -644,9 +644,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -684,7 +684,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -790,7 +790,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -932,7 +932,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -941,13 +941,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82FE0BB4-AF07-D248-8277-AD8E94C85802}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -967,7 +967,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -987,7 +987,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>50</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1047,7 +1047,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1081,7 +1081,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1163,12 +1163,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1957B83-55DF-0B40-AC0F-FC36128368F5}">
   <dimension ref="A1:K40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="5" width="17.83203125" customWidth="1"/>
+    <col min="7" max="7" width="6.5" customWidth="1"/>
+    <col min="8" max="8" width="19.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1185,7 +1187,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
@@ -1194,7 +1196,7 @@
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
@@ -1203,7 +1205,7 @@
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>7</v>
       </c>
@@ -1212,7 +1214,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -1221,7 +1223,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
@@ -1238,8 +1240,8 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="36" t="s">
         <v>10</v>
       </c>
@@ -1248,7 +1250,7 @@
       <c r="D8" s="37"/>
       <c r="E8" s="38"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>0</v>
       </c>
@@ -1265,7 +1267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>5</v>
       </c>
@@ -1274,7 +1276,7 @@
       <c r="D10" s="7"/>
       <c r="E10" s="11"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>6</v>
       </c>
@@ -1283,7 +1285,7 @@
       <c r="D11" s="7"/>
       <c r="E11" s="11"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>7</v>
       </c>
@@ -1292,7 +1294,7 @@
       <c r="D12" s="7"/>
       <c r="E12" s="11"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>8</v>
       </c>
@@ -1301,7 +1303,7 @@
       <c r="D13" s="7"/>
       <c r="E13" s="11"/>
     </row>
-    <row r="14" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="12" t="s">
         <v>9</v>
       </c>
@@ -1318,7 +1320,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="120" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="109" thickBot="1" x14ac:dyDescent="0.4">
       <c r="I16" s="15"/>
       <c r="J16" s="16" t="s">
         <v>20</v>
@@ -1327,7 +1329,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H17" s="42" t="s">
         <v>22</v>
       </c>
@@ -1341,7 +1343,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H18" s="43"/>
       <c r="I18" s="20" t="s">
         <v>24</v>
@@ -1353,7 +1355,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H19" s="43"/>
       <c r="I19" s="23" t="s">
         <v>27</v>
@@ -1365,7 +1367,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H20" s="43"/>
       <c r="I20" s="24" t="s">
         <v>30</v>
@@ -1377,7 +1379,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="8:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="8:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H21" s="44"/>
       <c r="I21" s="25" t="s">
         <v>33</v>
@@ -1389,7 +1391,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H22" s="42" t="s">
         <v>36</v>
       </c>
@@ -1403,7 +1405,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H23" s="43"/>
       <c r="I23" s="20" t="s">
         <v>24</v>
@@ -1415,7 +1417,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H24" s="43"/>
       <c r="I24" s="23" t="s">
         <v>27</v>
@@ -1427,7 +1429,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H25" s="43"/>
       <c r="I25" s="24" t="s">
         <v>30</v>
@@ -1439,7 +1441,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="8:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="8:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H26" s="44"/>
       <c r="I26" s="25" t="s">
         <v>33</v>
@@ -1451,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H27" s="42" t="s">
         <v>41</v>
       </c>
@@ -1465,7 +1467,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H28" s="43"/>
       <c r="I28" s="20" t="s">
         <v>24</v>
@@ -1477,7 +1479,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H29" s="43"/>
       <c r="I29" s="23" t="s">
         <v>27</v>
@@ -1489,7 +1491,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H30" s="43"/>
       <c r="I30" s="24" t="s">
         <v>30</v>
@@ -1501,7 +1503,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="8:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="8:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H31" s="44"/>
       <c r="I31" s="25" t="s">
         <v>33</v>
@@ -1513,7 +1515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H32" s="45" t="s">
         <v>43</v>
       </c>
@@ -1527,7 +1529,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H33" s="46"/>
       <c r="I33" s="20" t="s">
         <v>24</v>
@@ -1539,7 +1541,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H34" s="46"/>
       <c r="I34" s="23" t="s">
         <v>27</v>
@@ -1551,7 +1553,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H35" s="46"/>
       <c r="I35" s="24" t="s">
         <v>30</v>
@@ -1563,7 +1565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="8:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="8:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H36" s="47"/>
       <c r="I36" s="25" t="s">
         <v>33</v>
@@ -1575,7 +1577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H37" s="39" t="s">
         <v>45</v>
       </c>
@@ -1589,7 +1591,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H38" s="40"/>
       <c r="I38" s="23" t="s">
         <v>27</v>
@@ -1601,7 +1603,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="8:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="8:11" x14ac:dyDescent="0.35">
       <c r="H39" s="40"/>
       <c r="I39" s="24" t="s">
         <v>30</v>
@@ -1613,7 +1615,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="8:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="8:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H40" s="41"/>
       <c r="I40" s="25" t="s">
         <v>33</v>

</xml_diff>